<commit_message>
feat: Render v2 — botones de origen (Forma/SketchUp/Rhino) gobiernan el intro del JSON
Reemplaza los perfiles de atmósfera (Editorial/Comercial) por un selector de
"Origen del render": Forma / SketchUp / Rhino. Solo cambia el intro del JSON
(locked.role) — qué software produjo la imagen base —, no la atmósfera.

- Excel: nuevo param_key 'source' (3 filas, forma=default) con el prompt_en = intro.
- CondicionesToma.source; jsonBuilder: locked.role = prosa("source", toma.source)
  (antes hardcodeado "Forma color-coded massing…").
- PanelCondiciones: botones leen VOCAB.source, single-select, marcan el activo;
  se quitan los perfiles y sus props (perfiles/onPerfil).
- Textos de UI quedan genéricos (solo el JSON refleja el software elegido).

Verificado en Chrome: elegir SketchUp cambia locked.role a "SketchUp color-coded
massing…". tsc --noEmit limpio, build:config OK, master/copia del Excel en sync.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/config/render-config.xlsx
+++ b/frontend/config/render-config.xlsx
@@ -1624,7 +1624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6530,7 +6530,6 @@
           <t>preserve</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
           <t>geometria_camara</t>
@@ -6573,7 +6572,6 @@
           <t>preserve</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
           <t>contexto_blanco</t>
@@ -6616,7 +6614,6 @@
           <t>preserve</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>trazado_calles</t>
@@ -6659,7 +6656,6 @@
           <t>preserve</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
           <t>vegetacion_estructural</t>
@@ -6702,7 +6698,6 @@
           <t>preserve</t>
         </is>
       </c>
-      <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr">
         <is>
           <t>materiales_verticales</t>
@@ -6745,7 +6740,6 @@
           <t>avoid</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr">
         <is>
           <t>vegetacion_tropical</t>
@@ -6788,7 +6782,6 @@
           <t>avoid</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr">
         <is>
           <t>gloss_inmobiliario</t>
@@ -6814,6 +6807,123 @@
           <t>TRUE</t>
         </is>
       </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>locked.role</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>forma</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>render de Forma</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Autodesk Forma color-coded massing: each flat color is a USE, not a final material</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>locked.role</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>sketchup</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>render de SketchUp</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>SketchUp color-coded massing: each flat color is a USE, not a final material</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>locked.role</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>rhino</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>render de Rhino</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Rhino color-coded massing: each flat color is a USE, not a final material</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:H2"/>

</xml_diff>